<commit_message>
update: pricing and PDF templates
</commit_message>
<xml_diff>
--- a/Poster Pricing Config.xlsx
+++ b/Poster Pricing Config.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="146">
   <si>
     <t>Plan</t>
   </si>
@@ -211,55 +211,67 @@
     <t>eq_togo1</t>
   </si>
   <si>
-    <t>Комплект для точки to-go: планшет, принтер</t>
-  </si>
-  <si>
-    <t>eq_togo2</t>
-  </si>
-  <si>
-    <t>Комплект для точки to-go: планшет, принтер, підставка</t>
+    <t>Комплект для однієї каси: планшет та принтер</t>
   </si>
   <si>
     <t>eq_nowifi</t>
   </si>
   <si>
-    <t>Комплект для точки без інтернету (з SIM-картою)</t>
+    <t>Комплект з LTE планшетом та Bluetooth принтером</t>
   </si>
   <si>
     <t>eq_cafebar</t>
   </si>
   <si>
-    <t>Комплект для кафе та барів з деревʼяною підставкою</t>
+    <t>Комплект для закладу з кухнею</t>
   </si>
   <si>
-    <t>eq_lite</t>
+    <t>eq_shop1</t>
   </si>
   <si>
-    <t>Комплект обладнання Lite</t>
+    <t>Комплект для магазину з планшетом та вагами (без акумулятора)</t>
   </si>
   <si>
-    <t>eq_pro</t>
+    <t>eq_shop2</t>
   </si>
   <si>
-    <t>Комплект обладнання Pro</t>
+    <t>Комплект для магазину з планшетом та вагами (з акумулятором)</t>
   </si>
   <si>
-    <t>eq_shops</t>
+    <t>eq_shop3</t>
   </si>
   <si>
-    <t>Комплект для магазину з планшетом та вагами</t>
+    <t>Комплект для магазину з планшетом</t>
   </si>
   <si>
-    <t>eq_shopb</t>
+    <t>eq_shop4</t>
   </si>
   <si>
-    <t>Комплект POS обладнання для магазинів</t>
+    <t>Комплект для магазину з моноблоком та вагами без акумулятора</t>
   </si>
   <si>
-    <t>q260</t>
+    <t>eq_shop5</t>
   </si>
   <si>
-    <t>Принтер Xprinter Q260III</t>
+    <t>Комплект для магазину з моноблоком та вагами з акумулятором</t>
+  </si>
+  <si>
+    <t>eq_shop6</t>
+  </si>
+  <si>
+    <t>Комплект для магазину з моноблоком</t>
+  </si>
+  <si>
+    <t>sam_4s</t>
+  </si>
+  <si>
+    <t>Принтер Sam4S</t>
+  </si>
+  <si>
+    <t>xp_t890_b</t>
+  </si>
+  <si>
+    <t>Принтер Xprinter XP-Т890H Bluetooth</t>
   </si>
   <si>
     <t>xp_t890</t>
@@ -268,16 +280,10 @@
     <t>Принтер Xprinter XP-Т890H</t>
   </si>
   <si>
-    <t>xp_t890_b</t>
+    <t>q260</t>
   </si>
   <si>
-    <t>Принтер Xprinter XP-Т890H Bluetooth</t>
-  </si>
-  <si>
-    <t>sam_4s</t>
-  </si>
-  <si>
-    <t>Принтер Sam4S</t>
+    <t>Принтер Xprinter Q260III</t>
   </si>
   <si>
     <t>stand_w</t>
@@ -290,18 +296,6 @@
   </si>
   <si>
     <t>Універсальна металева підставка</t>
-  </si>
-  <si>
-    <t>cash_m</t>
-  </si>
-  <si>
-    <t>Грошова скринька середня</t>
-  </si>
-  <si>
-    <t>cahs_l</t>
-  </si>
-  <si>
-    <t>Грошова скринька велика</t>
   </si>
   <si>
     <t>pos_w</t>
@@ -322,16 +316,22 @@
     <t>Планшет iPad 10.2″ 64 GB 2021</t>
   </si>
   <si>
-    <t>taba9</t>
-  </si>
-  <si>
-    <t>Планшет Samsung Galaxy Tab A9 Plus Wi-Fi 4/64GB</t>
-  </si>
-  <si>
     <t>taba11</t>
   </si>
   <si>
     <t>Планшет Samsung Galaxy Tab A11+ 6/128GB Gray (WiFi)</t>
+  </si>
+  <si>
+    <t>cahs_l</t>
+  </si>
+  <si>
+    <t>Грошова скринька велика</t>
+  </si>
+  <si>
+    <t>cash_m</t>
+  </si>
+  <si>
+    <t>Грошова скринька середня</t>
   </si>
   <si>
     <t>rout_asus</t>
@@ -346,16 +346,16 @@
     <t>Cканер штрих-кодів</t>
   </si>
   <si>
-    <t>stand_scan</t>
+    <t>bta</t>
   </si>
   <si>
-    <t>Стійка (підставка) універсальна для сканерів штрихкодів</t>
+    <t>Ваги ВІС Промприлад з Ethernet</t>
   </si>
   <si>
-    <t>bta_60</t>
+    <t>bta_a</t>
   </si>
   <si>
-    <t>Ваги ВІС Промприлад BTA-60/15-5D-AC</t>
+    <t>Ваги ВІС Промприлад з Ethernet та акумулятором</t>
   </si>
   <si>
     <t>ring_k</t>
@@ -364,10 +364,28 @@
     <t>Дзвінок кухонний універсальний</t>
   </si>
   <si>
+    <t>stand_scan</t>
+  </si>
+  <si>
+    <t>Стійка (підставка) універсальна для сканерів штрихкодів</t>
+  </si>
+  <si>
     <t>roz_3_5</t>
   </si>
   <si>
     <t>Мережевий фільтр SPM5 3 метри 5 розеток</t>
+  </si>
+  <si>
+    <t>pospap3</t>
+  </si>
+  <si>
+    <t>Папір для чеків з логотипом Poster 3 шт.</t>
+  </si>
+  <si>
+    <t>pospap6</t>
+  </si>
+  <si>
+    <t>Папір для чеків з логотипом Poster 6 шт.</t>
   </si>
   <si>
     <t>pap_3</t>
@@ -391,13 +409,7 @@
     <t>pap_pos_3</t>
   </si>
   <si>
-    <t>Папір для чеків з логотипом Poster 3 шт.</t>
-  </si>
-  <si>
     <t>pap_pos_6</t>
-  </si>
-  <si>
-    <t>Папір для чеків з логотипом Poster 6 шт.</t>
   </si>
   <si>
     <t>lan_1</t>
@@ -493,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -538,13 +550,10 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
@@ -16292,7 +16301,7 @@
         <v>67</v>
       </c>
       <c r="C3" s="13">
-        <v>13500.0</v>
+        <v>16600.0</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -16303,7 +16312,7 @@
         <v>69</v>
       </c>
       <c r="C4" s="13">
-        <v>16600.0</v>
+        <v>17400.0</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -16314,29 +16323,29 @@
         <v>71</v>
       </c>
       <c r="C5" s="13">
-        <v>17400.0</v>
+        <v>23900.0</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="16">
-        <v>15895.0</v>
+      <c r="C6" s="13">
+        <v>24600.0</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="12" t="s">
         <v>75</v>
       </c>
       <c r="C7" s="13">
-        <v>25500.0</v>
+        <v>16700.0</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -16347,7 +16356,7 @@
         <v>77</v>
       </c>
       <c r="C8" s="13">
-        <v>23900.0</v>
+        <v>36000.0</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -16358,36 +16367,36 @@
         <v>79</v>
       </c>
       <c r="C9" s="13">
-        <v>33500.0</v>
+        <v>36700.0</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="16">
-        <v>3750.0</v>
+      <c r="C10" s="13">
+        <v>29500.0</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="15" t="s">
         <v>83</v>
       </c>
       <c r="C11" s="16">
-        <v>4995.0</v>
+        <v>7400.0</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="15" t="s">
         <v>85</v>
       </c>
       <c r="C12" s="16">
@@ -16398,29 +16407,29 @@
       <c r="A13" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="15" t="s">
         <v>87</v>
       </c>
       <c r="C13" s="16">
-        <v>7400.0</v>
+        <v>4995.0</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="15" t="s">
         <v>89</v>
       </c>
       <c r="C14" s="16">
-        <v>950.0</v>
+        <v>3750.0</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="15" t="s">
         <v>91</v>
       </c>
       <c r="C15" s="16">
@@ -16431,29 +16440,29 @@
       <c r="A16" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="15" t="s">
         <v>93</v>
       </c>
       <c r="C16" s="16">
-        <v>2100.0</v>
+        <v>950.0</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="15" t="s">
         <v>95</v>
       </c>
       <c r="C17" s="16">
-        <v>2400.0</v>
+        <v>22990.0</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="15" t="s">
         <v>97</v>
       </c>
       <c r="C18" s="16">
@@ -16464,51 +16473,51 @@
       <c r="A19" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="15" t="s">
         <v>99</v>
       </c>
       <c r="C19" s="16">
-        <v>22990.0</v>
+        <v>17000.0</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="11" t="s">
         <v>100</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="16">
-        <v>17000.0</v>
+      <c r="C20" s="13">
+        <v>10200.0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="15" t="s">
         <v>103</v>
       </c>
       <c r="C21" s="16">
-        <v>9800.0</v>
+        <v>2400.0</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="13">
-        <v>10200.0</v>
+      <c r="C22" s="16">
+        <v>2100.0</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="15" t="s">
         <v>107</v>
       </c>
       <c r="C23" s="16">
@@ -16519,7 +16528,7 @@
       <c r="A24" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="17" t="s">
         <v>109</v>
       </c>
       <c r="C24" s="16">
@@ -16527,32 +16536,32 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="11" t="s">
         <v>110</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>111</v>
       </c>
       <c r="C25" s="16">
-        <v>400.0</v>
+        <v>6590.0</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="C26" s="16">
-        <v>6590.0</v>
+      <c r="C26" s="18">
+        <v>7290.0</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="15" t="s">
         <v>115</v>
       </c>
       <c r="C27" s="16">
@@ -16563,18 +16572,18 @@
       <c r="A28" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="15" t="s">
         <v>117</v>
       </c>
       <c r="C28" s="16">
-        <v>350.0</v>
+        <v>400.0</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="15" t="s">
         <v>119</v>
       </c>
       <c r="C29" s="16">
@@ -16582,917 +16591,947 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="16">
-        <v>900.0</v>
+      <c r="C30" s="18">
+        <v>300.0</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="18" t="s">
         <v>122</v>
       </c>
       <c r="B31" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="C31" s="13">
-        <v>2100.0</v>
+      <c r="C31" s="18">
+        <v>580.0</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="15" t="s">
         <v>125</v>
       </c>
       <c r="C32" s="16">
-        <v>300.0</v>
+        <v>350.0</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="15" t="s">
         <v>127</v>
       </c>
       <c r="C33" s="16">
-        <v>580.0</v>
+        <v>900.0</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="14" t="s">
+      <c r="A34" s="11" t="s">
         <v>128</v>
       </c>
       <c r="B34" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="C34" s="16">
-        <v>150.0</v>
+      <c r="C34" s="13">
+        <v>2100.0</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="B35" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="C35" s="13">
+      <c r="B35" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C35" s="16">
         <v>300.0</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="C36" s="13">
-        <v>400.0</v>
+        <v>131</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C36" s="16">
+        <v>580.0</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C37" s="16">
+        <v>150.0</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B38" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C37" s="13">
+      <c r="C38" s="13">
+        <v>300.0</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="C39" s="13">
+        <v>400.0</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="C40" s="13">
         <v>500.0</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="B38" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="C38" s="18">
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C41" s="17">
         <v>600.0</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="B39" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="C39" s="18">
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="C42" s="17">
         <v>800.0</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="B40" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="C40" s="18">
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C43" s="17">
         <v>1000.0</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-    </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="B46" s="17"/>
-      <c r="C46" s="17"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="B50" s="17"/>
-      <c r="C50" s="17"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="B51" s="17"/>
-      <c r="C51" s="17"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="B57" s="17"/>
-      <c r="C57" s="17"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="15"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="B60" s="17"/>
-      <c r="C60" s="17"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="B61" s="17"/>
-      <c r="C61" s="17"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="B62" s="17"/>
-      <c r="C62" s="17"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="B63" s="17"/>
-      <c r="C63" s="17"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="B64" s="17"/>
-      <c r="C64" s="17"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="B65" s="17"/>
-      <c r="C65" s="17"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="B67" s="17"/>
-      <c r="C67" s="17"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="15"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="B68" s="17"/>
-      <c r="C68" s="17"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="15"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="B69" s="17"/>
-      <c r="C69" s="17"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="15"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="15"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="B71" s="17"/>
-      <c r="C71" s="17"/>
+      <c r="B71" s="15"/>
+      <c r="C71" s="15"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="B72" s="17"/>
-      <c r="C72" s="17"/>
+      <c r="B72" s="15"/>
+      <c r="C72" s="15"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="B73" s="17"/>
-      <c r="C73" s="17"/>
+      <c r="B73" s="15"/>
+      <c r="C73" s="15"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="B74" s="17"/>
-      <c r="C74" s="17"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="15"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="B75" s="17"/>
-      <c r="C75" s="17"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="15"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="B76" s="17"/>
-      <c r="C76" s="17"/>
+      <c r="B76" s="15"/>
+      <c r="C76" s="15"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="B77" s="17"/>
-      <c r="C77" s="17"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="15"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="B78" s="17"/>
-      <c r="C78" s="17"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="15"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="B79" s="17"/>
-      <c r="C79" s="17"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="15"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="B80" s="17"/>
-      <c r="C80" s="17"/>
+      <c r="B80" s="15"/>
+      <c r="C80" s="15"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="B81" s="17"/>
-      <c r="C81" s="17"/>
+      <c r="B81" s="15"/>
+      <c r="C81" s="15"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="B82" s="17"/>
-      <c r="C82" s="17"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="15"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="B83" s="17"/>
-      <c r="C83" s="17"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="15"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="B84" s="17"/>
-      <c r="C84" s="17"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="15"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="B85" s="17"/>
-      <c r="C85" s="17"/>
+      <c r="B85" s="15"/>
+      <c r="C85" s="15"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="B86" s="17"/>
-      <c r="C86" s="17"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="15"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="B87" s="17"/>
-      <c r="C87" s="17"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="15"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="B88" s="17"/>
-      <c r="C88" s="17"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="15"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="B89" s="17"/>
-      <c r="C89" s="17"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="15"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="B90" s="17"/>
-      <c r="C90" s="17"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="15"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="B91" s="17"/>
-      <c r="C91" s="17"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="15"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="B92" s="17"/>
-      <c r="C92" s="17"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="15"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="B93" s="17"/>
-      <c r="C93" s="17"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="15"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="B94" s="17"/>
-      <c r="C94" s="17"/>
+      <c r="B94" s="15"/>
+      <c r="C94" s="15"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="B95" s="17"/>
-      <c r="C95" s="17"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="15"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="B96" s="17"/>
-      <c r="C96" s="17"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="15"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="B97" s="17"/>
-      <c r="C97" s="17"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="15"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="B98" s="17"/>
-      <c r="C98" s="17"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="15"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="B99" s="17"/>
-      <c r="C99" s="17"/>
+      <c r="B99" s="15"/>
+      <c r="C99" s="15"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
-      <c r="B100" s="17"/>
-      <c r="C100" s="17"/>
+      <c r="B100" s="15"/>
+      <c r="C100" s="15"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
-      <c r="B101" s="17"/>
-      <c r="C101" s="17"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="15"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="B102" s="17"/>
-      <c r="C102" s="17"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="15"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="B103" s="17"/>
-      <c r="C103" s="17"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="15"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="B104" s="17"/>
-      <c r="C104" s="17"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="15"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="B105" s="17"/>
-      <c r="C105" s="17"/>
+      <c r="B105" s="15"/>
+      <c r="C105" s="15"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="B106" s="17"/>
-      <c r="C106" s="17"/>
+      <c r="B106" s="15"/>
+      <c r="C106" s="15"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="B107" s="17"/>
-      <c r="C107" s="17"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="15"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="B108" s="17"/>
-      <c r="C108" s="17"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="15"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="B109" s="17"/>
-      <c r="C109" s="17"/>
+      <c r="B109" s="15"/>
+      <c r="C109" s="15"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="B110" s="17"/>
-      <c r="C110" s="17"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="15"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="B111" s="17"/>
-      <c r="C111" s="17"/>
+      <c r="B111" s="15"/>
+      <c r="C111" s="15"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="B112" s="17"/>
-      <c r="C112" s="17"/>
+      <c r="B112" s="15"/>
+      <c r="C112" s="15"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="B113" s="17"/>
-      <c r="C113" s="17"/>
+      <c r="B113" s="15"/>
+      <c r="C113" s="15"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="B114" s="17"/>
-      <c r="C114" s="17"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="15"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="B115" s="17"/>
-      <c r="C115" s="17"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="15"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="B116" s="17"/>
-      <c r="C116" s="17"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="15"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="B117" s="17"/>
-      <c r="C117" s="17"/>
+      <c r="B117" s="15"/>
+      <c r="C117" s="15"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
-      <c r="B118" s="17"/>
-      <c r="C118" s="17"/>
+      <c r="B118" s="15"/>
+      <c r="C118" s="15"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="B119" s="17"/>
-      <c r="C119" s="17"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="15"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="B120" s="17"/>
-      <c r="C120" s="17"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="15"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="B121" s="17"/>
-      <c r="C121" s="17"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="15"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
-      <c r="B122" s="17"/>
-      <c r="C122" s="17"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="15"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
-      <c r="B123" s="17"/>
-      <c r="C123" s="17"/>
+      <c r="B123" s="15"/>
+      <c r="C123" s="15"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
-      <c r="B124" s="17"/>
-      <c r="C124" s="17"/>
+      <c r="B124" s="15"/>
+      <c r="C124" s="15"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
-      <c r="B125" s="17"/>
-      <c r="C125" s="17"/>
+      <c r="B125" s="15"/>
+      <c r="C125" s="15"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
-      <c r="B126" s="17"/>
-      <c r="C126" s="17"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="15"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
-      <c r="B127" s="17"/>
-      <c r="C127" s="17"/>
+      <c r="B127" s="15"/>
+      <c r="C127" s="15"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
-      <c r="B128" s="17"/>
-      <c r="C128" s="17"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="15"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
-      <c r="B129" s="17"/>
-      <c r="C129" s="17"/>
+      <c r="B129" s="15"/>
+      <c r="C129" s="15"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
-      <c r="B130" s="17"/>
-      <c r="C130" s="17"/>
+      <c r="B130" s="15"/>
+      <c r="C130" s="15"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
-      <c r="B131" s="17"/>
-      <c r="C131" s="17"/>
+      <c r="B131" s="15"/>
+      <c r="C131" s="15"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
-      <c r="B132" s="17"/>
-      <c r="C132" s="17"/>
+      <c r="B132" s="15"/>
+      <c r="C132" s="15"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
-      <c r="B133" s="17"/>
-      <c r="C133" s="17"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="15"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
-      <c r="B134" s="17"/>
-      <c r="C134" s="17"/>
+      <c r="B134" s="15"/>
+      <c r="C134" s="15"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
-      <c r="B135" s="17"/>
-      <c r="C135" s="17"/>
+      <c r="B135" s="15"/>
+      <c r="C135" s="15"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
-      <c r="B136" s="17"/>
-      <c r="C136" s="17"/>
+      <c r="B136" s="15"/>
+      <c r="C136" s="15"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
-      <c r="B137" s="17"/>
-      <c r="C137" s="17"/>
+      <c r="B137" s="15"/>
+      <c r="C137" s="15"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
-      <c r="B138" s="17"/>
-      <c r="C138" s="17"/>
+      <c r="B138" s="15"/>
+      <c r="C138" s="15"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
-      <c r="B139" s="17"/>
-      <c r="C139" s="17"/>
+      <c r="B139" s="15"/>
+      <c r="C139" s="15"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="B140" s="17"/>
-      <c r="C140" s="17"/>
+      <c r="B140" s="15"/>
+      <c r="C140" s="15"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="B141" s="17"/>
-      <c r="C141" s="17"/>
+      <c r="B141" s="15"/>
+      <c r="C141" s="15"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="B142" s="17"/>
-      <c r="C142" s="17"/>
+      <c r="B142" s="15"/>
+      <c r="C142" s="15"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="B143" s="17"/>
-      <c r="C143" s="17"/>
+      <c r="B143" s="15"/>
+      <c r="C143" s="15"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="B144" s="17"/>
-      <c r="C144" s="17"/>
+      <c r="B144" s="15"/>
+      <c r="C144" s="15"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="B145" s="17"/>
-      <c r="C145" s="17"/>
+      <c r="B145" s="15"/>
+      <c r="C145" s="15"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="B146" s="17"/>
-      <c r="C146" s="17"/>
+      <c r="B146" s="15"/>
+      <c r="C146" s="15"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="B147" s="17"/>
-      <c r="C147" s="17"/>
+      <c r="B147" s="15"/>
+      <c r="C147" s="15"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="B148" s="17"/>
-      <c r="C148" s="17"/>
+      <c r="B148" s="15"/>
+      <c r="C148" s="15"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="B149" s="17"/>
-      <c r="C149" s="17"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="B150" s="17"/>
-      <c r="C150" s="17"/>
+      <c r="B150" s="15"/>
+      <c r="C150" s="15"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="B151" s="17"/>
-      <c r="C151" s="17"/>
+      <c r="B151" s="15"/>
+      <c r="C151" s="15"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="B152" s="17"/>
-      <c r="C152" s="17"/>
+      <c r="B152" s="15"/>
+      <c r="C152" s="15"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="B153" s="17"/>
-      <c r="C153" s="17"/>
+      <c r="B153" s="15"/>
+      <c r="C153" s="15"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="B154" s="17"/>
-      <c r="C154" s="17"/>
+      <c r="B154" s="15"/>
+      <c r="C154" s="15"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="B155" s="17"/>
-      <c r="C155" s="17"/>
+      <c r="B155" s="15"/>
+      <c r="C155" s="15"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="B156" s="17"/>
-      <c r="C156" s="17"/>
+      <c r="B156" s="15"/>
+      <c r="C156" s="15"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="B157" s="17"/>
-      <c r="C157" s="17"/>
+      <c r="B157" s="15"/>
+      <c r="C157" s="15"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
-      <c r="B158" s="17"/>
-      <c r="C158" s="17"/>
+      <c r="B158" s="15"/>
+      <c r="C158" s="15"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="B159" s="17"/>
-      <c r="C159" s="17"/>
+      <c r="B159" s="15"/>
+      <c r="C159" s="15"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
-      <c r="B160" s="17"/>
-      <c r="C160" s="17"/>
+      <c r="B160" s="15"/>
+      <c r="C160" s="15"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="B161" s="17"/>
-      <c r="C161" s="17"/>
+      <c r="B161" s="15"/>
+      <c r="C161" s="15"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
-      <c r="B162" s="17"/>
-      <c r="C162" s="17"/>
+      <c r="B162" s="15"/>
+      <c r="C162" s="15"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
-      <c r="B163" s="17"/>
-      <c r="C163" s="17"/>
+      <c r="B163" s="15"/>
+      <c r="C163" s="15"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="B164" s="17"/>
-      <c r="C164" s="17"/>
+      <c r="B164" s="15"/>
+      <c r="C164" s="15"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
-      <c r="B165" s="17"/>
-      <c r="C165" s="17"/>
+      <c r="B165" s="15"/>
+      <c r="C165" s="15"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
-      <c r="B166" s="17"/>
-      <c r="C166" s="17"/>
+      <c r="B166" s="15"/>
+      <c r="C166" s="15"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
-      <c r="B167" s="17"/>
-      <c r="C167" s="17"/>
+      <c r="B167" s="15"/>
+      <c r="C167" s="15"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
-      <c r="B168" s="17"/>
-      <c r="C168" s="17"/>
+      <c r="B168" s="15"/>
+      <c r="C168" s="15"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="B169" s="17"/>
-      <c r="C169" s="17"/>
+      <c r="B169" s="15"/>
+      <c r="C169" s="15"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="B170" s="17"/>
-      <c r="C170" s="17"/>
+      <c r="B170" s="15"/>
+      <c r="C170" s="15"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="B171" s="17"/>
-      <c r="C171" s="17"/>
+      <c r="B171" s="15"/>
+      <c r="C171" s="15"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="B172" s="17"/>
-      <c r="C172" s="17"/>
+      <c r="B172" s="15"/>
+      <c r="C172" s="15"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
-      <c r="B173" s="17"/>
-      <c r="C173" s="17"/>
+      <c r="B173" s="15"/>
+      <c r="C173" s="15"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="B174" s="17"/>
-      <c r="C174" s="17"/>
+      <c r="B174" s="15"/>
+      <c r="C174" s="15"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="B175" s="17"/>
-      <c r="C175" s="17"/>
+      <c r="B175" s="15"/>
+      <c r="C175" s="15"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="B176" s="17"/>
-      <c r="C176" s="17"/>
+      <c r="B176" s="15"/>
+      <c r="C176" s="15"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="B177" s="17"/>
-      <c r="C177" s="17"/>
+      <c r="B177" s="15"/>
+      <c r="C177" s="15"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="B178" s="17"/>
-      <c r="C178" s="17"/>
+      <c r="B178" s="15"/>
+      <c r="C178" s="15"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="B179" s="17"/>
-      <c r="C179" s="17"/>
+      <c r="B179" s="15"/>
+      <c r="C179" s="15"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
-      <c r="B180" s="17"/>
-      <c r="C180" s="17"/>
+      <c r="B180" s="15"/>
+      <c r="C180" s="15"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
-      <c r="B181" s="17"/>
-      <c r="C181" s="17"/>
+      <c r="B181" s="15"/>
+      <c r="C181" s="15"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
-      <c r="B182" s="17"/>
-      <c r="C182" s="17"/>
+      <c r="B182" s="15"/>
+      <c r="C182" s="15"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
-      <c r="B183" s="17"/>
-      <c r="C183" s="17"/>
+      <c r="B183" s="15"/>
+      <c r="C183" s="15"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
-      <c r="B184" s="17"/>
-      <c r="C184" s="17"/>
+      <c r="B184" s="15"/>
+      <c r="C184" s="15"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
-      <c r="B185" s="17"/>
-      <c r="C185" s="17"/>
+      <c r="B185" s="15"/>
+      <c r="C185" s="15"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
-      <c r="B186" s="17"/>
-      <c r="C186" s="17"/>
+      <c r="B186" s="15"/>
+      <c r="C186" s="15"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
-      <c r="B187" s="17"/>
-      <c r="C187" s="17"/>
+      <c r="B187" s="15"/>
+      <c r="C187" s="15"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
-      <c r="B188" s="17"/>
-      <c r="C188" s="17"/>
+      <c r="B188" s="15"/>
+      <c r="C188" s="15"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
-      <c r="B189" s="17"/>
-      <c r="C189" s="17"/>
+      <c r="B189" s="15"/>
+      <c r="C189" s="15"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
-      <c r="B190" s="17"/>
-      <c r="C190" s="17"/>
+      <c r="B190" s="15"/>
+      <c r="C190" s="15"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
-      <c r="B191" s="17"/>
-      <c r="C191" s="17"/>
+      <c r="B191" s="15"/>
+      <c r="C191" s="15"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
-      <c r="B192" s="17"/>
-      <c r="C192" s="17"/>
+      <c r="B192" s="15"/>
+      <c r="C192" s="15"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
-      <c r="B193" s="17"/>
-      <c r="C193" s="17"/>
+      <c r="B193" s="15"/>
+      <c r="C193" s="15"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
-      <c r="B194" s="17"/>
-      <c r="C194" s="17"/>
+      <c r="B194" s="15"/>
+      <c r="C194" s="15"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="B195" s="17"/>
-      <c r="C195" s="17"/>
+      <c r="B195" s="15"/>
+      <c r="C195" s="15"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="B196" s="17"/>
-      <c r="C196" s="17"/>
+      <c r="B196" s="15"/>
+      <c r="C196" s="15"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="B197" s="17"/>
-      <c r="C197" s="17"/>
+      <c r="B197" s="15"/>
+      <c r="C197" s="15"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="B198" s="17"/>
-      <c r="C198" s="17"/>
+      <c r="B198" s="15"/>
+      <c r="C198" s="15"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="B199" s="17"/>
-      <c r="C199" s="17"/>
+      <c r="B199" s="15"/>
+      <c r="C199" s="15"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
-      <c r="B200" s="17"/>
-      <c r="C200" s="17"/>
+      <c r="B200" s="15"/>
+      <c r="C200" s="15"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
-      <c r="B201" s="17"/>
-      <c r="C201" s="17"/>
+      <c r="B201" s="15"/>
+      <c r="C201" s="15"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
-      <c r="B202" s="17"/>
-      <c r="C202" s="17"/>
+      <c r="B202" s="15"/>
+      <c r="C202" s="15"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="B203" s="17"/>
-      <c r="C203" s="17"/>
+      <c r="B203" s="15"/>
+      <c r="C203" s="15"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
-      <c r="B204" s="17"/>
-      <c r="C204" s="17"/>
+      <c r="B204" s="15"/>
+      <c r="C204" s="15"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
-      <c r="B205" s="17"/>
-      <c r="C205" s="17"/>
+      <c r="B205" s="15"/>
+      <c r="C205" s="15"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
-      <c r="B206" s="17"/>
-      <c r="C206" s="17"/>
+      <c r="B206" s="15"/>
+      <c r="C206" s="15"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
-      <c r="B207" s="17"/>
-      <c r="C207" s="17"/>
+      <c r="B207" s="15"/>
+      <c r="C207" s="15"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
-      <c r="B208" s="17"/>
-      <c r="C208" s="17"/>
+      <c r="B208" s="15"/>
+      <c r="C208" s="15"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
-      <c r="B209" s="17"/>
-      <c r="C209" s="17"/>
+      <c r="B209" s="15"/>
+      <c r="C209" s="15"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
-      <c r="B210" s="17"/>
-      <c r="C210" s="17"/>
+      <c r="B210" s="15"/>
+      <c r="C210" s="15"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="B211" s="17"/>
-      <c r="C211" s="17"/>
+      <c r="B211" s="15"/>
+      <c r="C211" s="15"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
-      <c r="B212" s="17"/>
-      <c r="C212" s="17"/>
+      <c r="B212" s="15"/>
+      <c r="C212" s="15"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="B213" s="17"/>
-      <c r="C213" s="17"/>
+      <c r="B213" s="15"/>
+      <c r="C213" s="15"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
-      <c r="B214" s="17"/>
-      <c r="C214" s="17"/>
+      <c r="B214" s="15"/>
+      <c r="C214" s="15"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="B215" s="17"/>
-      <c r="C215" s="17"/>
+      <c r="B215" s="15"/>
+      <c r="C215" s="15"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
-      <c r="B216" s="17"/>
-      <c r="C216" s="17"/>
+      <c r="B216" s="15"/>
+      <c r="C216" s="15"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
-      <c r="B217" s="17"/>
-      <c r="C217" s="17"/>
+      <c r="B217" s="15"/>
+      <c r="C217" s="15"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="B218" s="17"/>
-      <c r="C218" s="17"/>
+      <c r="B218" s="15"/>
+      <c r="C218" s="15"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="B219" s="17"/>
-      <c r="C219" s="17"/>
+      <c r="B219" s="15"/>
+      <c r="C219" s="15"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
-      <c r="B220" s="17"/>
-      <c r="C220" s="17"/>
+      <c r="B220" s="15"/>
+      <c r="C220" s="15"/>
     </row>
     <row r="221" ht="15.75" customHeight="1">
-      <c r="B221" s="17"/>
-      <c r="C221" s="17"/>
+      <c r="B221" s="15"/>
+      <c r="C221" s="15"/>
     </row>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="B222" s="17"/>
-      <c r="C222" s="17"/>
+      <c r="B222" s="15"/>
+      <c r="C222" s="15"/>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="B223" s="17"/>
-      <c r="C223" s="17"/>
+      <c r="B223" s="15"/>
+      <c r="C223" s="15"/>
     </row>
     <row r="224" ht="15.75" customHeight="1">
-      <c r="B224" s="17"/>
-      <c r="C224" s="17"/>
+      <c r="B224" s="15"/>
+      <c r="C224" s="15"/>
     </row>
     <row r="225" ht="15.75" customHeight="1">
-      <c r="B225" s="17"/>
-      <c r="C225" s="17"/>
+      <c r="B225" s="15"/>
+      <c r="C225" s="15"/>
     </row>
     <row r="226" ht="15.75" customHeight="1">
-      <c r="B226" s="17"/>
-      <c r="C226" s="17"/>
+      <c r="B226" s="15"/>
+      <c r="C226" s="15"/>
     </row>
     <row r="227" ht="15.75" customHeight="1">
-      <c r="B227" s="17"/>
-      <c r="C227" s="17"/>
+      <c r="B227" s="15"/>
+      <c r="C227" s="15"/>
     </row>
     <row r="228" ht="15.75" customHeight="1">
-      <c r="B228" s="17"/>
-      <c r="C228" s="17"/>
+      <c r="B228" s="15"/>
+      <c r="C228" s="15"/>
     </row>
     <row r="229" ht="15.75" customHeight="1">
-      <c r="B229" s="17"/>
-      <c r="C229" s="17"/>
+      <c r="B229" s="15"/>
+      <c r="C229" s="15"/>
     </row>
     <row r="230" ht="15.75" customHeight="1">
-      <c r="B230" s="17"/>
-      <c r="C230" s="17"/>
+      <c r="B230" s="15"/>
+      <c r="C230" s="15"/>
     </row>
     <row r="231" ht="15.75" customHeight="1">
-      <c r="B231" s="17"/>
-      <c r="C231" s="17"/>
+      <c r="B231" s="15"/>
+      <c r="C231" s="15"/>
     </row>
     <row r="232" ht="15.75" customHeight="1">
-      <c r="B232" s="17"/>
-      <c r="C232" s="17"/>
+      <c r="B232" s="15"/>
+      <c r="C232" s="15"/>
     </row>
     <row r="233" ht="15.75" customHeight="1">
-      <c r="B233" s="17"/>
-      <c r="C233" s="17"/>
+      <c r="B233" s="15"/>
+      <c r="C233" s="15"/>
     </row>
     <row r="234" ht="15.75" customHeight="1">
-      <c r="B234" s="17"/>
-      <c r="C234" s="17"/>
+      <c r="B234" s="15"/>
+      <c r="C234" s="15"/>
     </row>
     <row r="235" ht="15.75" customHeight="1">
-      <c r="B235" s="17"/>
-      <c r="C235" s="17"/>
+      <c r="B235" s="15"/>
+      <c r="C235" s="15"/>
     </row>
     <row r="236" ht="15.75" customHeight="1">
-      <c r="B236" s="17"/>
-      <c r="C236" s="17"/>
+      <c r="B236" s="15"/>
+      <c r="C236" s="15"/>
     </row>
     <row r="237" ht="15.75" customHeight="1">
-      <c r="B237" s="17"/>
-      <c r="C237" s="17"/>
-    </row>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
+      <c r="B237" s="15"/>
+      <c r="C237" s="15"/>
+    </row>
+    <row r="238" ht="15.75" customHeight="1">
+      <c r="B238" s="15"/>
+      <c r="C238" s="15"/>
+    </row>
+    <row r="239" ht="15.75" customHeight="1">
+      <c r="B239" s="15"/>
+      <c r="C239" s="15"/>
+    </row>
+    <row r="240" ht="15.75" customHeight="1">
+      <c r="B240" s="15"/>
+      <c r="C240" s="15"/>
+    </row>
     <row r="241" ht="15.75" customHeight="1"/>
     <row r="242" ht="15.75" customHeight="1"/>
     <row r="243" ht="15.75" customHeight="1"/>
@@ -18253,6 +18292,9 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>